<commit_message>
Finalize duplicate-pair redirects: direction in tracker + ready rules
Set Final Decision/Notes in the OP-02 Blog Audit tab for all 8 rows in
the 4 duplicate pairs - each winner marked Keep (with the click/position
data behind the call), each loser marked Merge/301 with the explicit
destination URL, so the tab itself now carries the answer rather than
just flagging "these are duplicates."

Drafted docs/seo/technical/OP-02-duplicate-redirects.md: a Rank Math
Redirections table (recommended, since Rank Math is already installed)
and a raw .htaccess fallback, both ready to paste in. Repeated the
merge-content-first caveat - a 301 moves the URL's authority, not its
text.

Not applied - needs WordPress/hosting access this agent doesn't have.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VmvRFCrr5iCSGjZGbzZndE
</commit_message>
<xml_diff>
--- a/docs/seo/DrRanaIrfanSEOIssueTracker.xlsx
+++ b/docs/seo/DrRanaIrfanSEOIssueTracker.xlsx
@@ -56193,7 +56193,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G11"/>
+  <dimension ref="A1:G12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" style="23" min="1" max="1"/>
@@ -56486,6 +56486,43 @@
         </is>
       </c>
       <c r="G11" s="32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="120" customHeight="1" s="23">
+      <c r="A12" s="31" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B12" s="31" t="inlineStr">
+        <is>
+          <t>On Page SEO Issue</t>
+        </is>
+      </c>
+      <c r="C12" s="31" t="inlineStr">
+        <is>
+          <t>OP-02 (4 duplicate pairs)</t>
+        </is>
+      </c>
+      <c r="D12" s="31" t="inlineStr">
+        <is>
+          <t>Finalized the redirect direction for the 4 duplicate/near-duplicate pairs found in the OP-02 blog audit, and drafted the actual redirect rules ready to apply.</t>
+        </is>
+      </c>
+      <c r="E12" s="31" t="inlineStr">
+        <is>
+          <t>Set Final Decision/Notes in the 'OP-02 Blog Audit' tab for all 8 rows in the 4 pairs - each winner marked Keep (with why), each loser marked Merge/301 with the explicit destination URL. Wrote both a Rank Math Redirections table and raw .htaccess RewriteRule syntax in docs/seo/technical/OP-02-duplicate-redirects.md, with the merge-content-first caveat repeated. Did not apply any redirect - needs WordPress/hosting access this agent doesn't have.</t>
+        </is>
+      </c>
+      <c r="F12" s="31" t="inlineStr">
+        <is>
+          <t>DrRanaIrfanSEOIssueTracker.xlsx tab 'OP-02 Blog Audit' (8 rows); docs/seo/technical/OP-02-duplicate-redirects.md</t>
+        </is>
+      </c>
+      <c r="G12" s="32" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -56512,7 +56549,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J255"/>
+  <dimension ref="A1:J259"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="46" customWidth="1" style="23" min="1" max="1"/>
@@ -56917,9 +56954,17 @@
           <t>Merge/301</t>
         </is>
       </c>
-      <c r="H14" s="38" t="n"/>
+      <c r="H14" s="38" t="inlineStr">
+        <is>
+          <t>Merge/301</t>
+        </is>
+      </c>
       <c r="I14" s="38" t="n"/>
-      <c r="J14" s="38" t="n"/>
+      <c r="J14" s="38" t="inlineStr">
+        <is>
+          <t>301 THIS -&gt; /how-much-does-hair-weigh/ (keep the winner: 48 clicks/90d vs 36, better position 6.1 vs 7.1 despite more impressions here). Merge any unique content into the winner first. Redirect rule drafted in docs/seo/technical/OP-02-duplicate-redirects.md.</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="33" t="inlineStr">
@@ -57109,9 +57154,17 @@
           <t>Merge/301</t>
         </is>
       </c>
-      <c r="H20" s="38" t="n"/>
+      <c r="H20" s="38" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="I20" s="38" t="n"/>
-      <c r="J20" s="38" t="n"/>
+      <c r="J20" s="38" t="inlineStr">
+        <is>
+          <t>KEEP as the 301 destination for /does-hair-weigh-anything/ (48 clicks/90d vs 36, better position).</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="33" t="inlineStr">
@@ -58773,9 +58826,17 @@
           <t>Merge/301</t>
         </is>
       </c>
-      <c r="H72" s="38" t="n"/>
+      <c r="H72" s="38" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="I72" s="38" t="n"/>
-      <c r="J72" s="38" t="n"/>
+      <c r="J72" s="38" t="inlineStr">
+        <is>
+          <t>KEEP as the 301 destination for /does-zyn-cause-hair-loss/ (50 clicks/90d vs 25 - the '-2' URL is the stronger one).</t>
+        </is>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="33" t="inlineStr">
@@ -59285,9 +59346,17 @@
           <t>Merge/301</t>
         </is>
       </c>
-      <c r="H88" s="38" t="n"/>
+      <c r="H88" s="38" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="I88" s="38" t="n"/>
-      <c r="J88" s="38" t="n"/>
+      <c r="J88" s="38" t="inlineStr">
+        <is>
+          <t>KEEP as the 301 destination for /can-low-blood-pressure-cause-hair-loss/ (79 clicks/90d vs 8 - clear winner).</t>
+        </is>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="33" t="inlineStr">
@@ -59733,9 +59802,17 @@
           <t>Merge/301</t>
         </is>
       </c>
-      <c r="H102" s="38" t="n"/>
+      <c r="H102" s="38" t="inlineStr">
+        <is>
+          <t>Merge/301</t>
+        </is>
+      </c>
       <c r="I102" s="38" t="n"/>
-      <c r="J102" s="38" t="n"/>
+      <c r="J102" s="38" t="inlineStr">
+        <is>
+          <t>301 THIS -&gt; /does-zyn-cause-hair-loss-2/ (keep the winner: 50 clicks/90d vs 25, despite the uglier '-2' slug - don't rename it, that just creates another redirect to manage). Merge any unique content into the winner first. Redirect rule drafted in docs/seo/technical/OP-02-duplicate-redirects.md.</t>
+        </is>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="33" t="inlineStr">
@@ -59861,9 +59938,17 @@
           <t>Merge/301</t>
         </is>
       </c>
-      <c r="H106" s="38" t="n"/>
+      <c r="H106" s="38" t="inlineStr">
+        <is>
+          <t>Keep</t>
+        </is>
+      </c>
       <c r="I106" s="38" t="n"/>
-      <c r="J106" s="38" t="n"/>
+      <c r="J106" s="38" t="inlineStr">
+        <is>
+          <t>KEEP as the 301 destination for /title-can-progesterone-cause-hair-loss/ (15 clicks/90d vs 6 - clear winner).</t>
+        </is>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="33" t="inlineStr">
@@ -60853,9 +60938,17 @@
           <t>Merge/301</t>
         </is>
       </c>
-      <c r="H137" s="38" t="n"/>
+      <c r="H137" s="38" t="inlineStr">
+        <is>
+          <t>Merge/301</t>
+        </is>
+      </c>
       <c r="I137" s="38" t="n"/>
-      <c r="J137" s="38" t="n"/>
+      <c r="J137" s="38" t="inlineStr">
+        <is>
+          <t>301 THIS -&gt; /progesterone-female-hair-loss/ (keep the winner: 15 clicks/90d vs 6; this slug also still carries a leftover 'title-' prefix from a bad import). Merge any unique content into the winner first. Redirect rule drafted in docs/seo/technical/OP-02-duplicate-redirects.md.</t>
+        </is>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="33" t="inlineStr">
@@ -61653,9 +61746,17 @@
           <t>Merge/301</t>
         </is>
       </c>
-      <c r="H162" s="38" t="n"/>
+      <c r="H162" s="38" t="inlineStr">
+        <is>
+          <t>Merge/301</t>
+        </is>
+      </c>
       <c r="I162" s="38" t="n"/>
-      <c r="J162" s="38" t="n"/>
+      <c r="J162" s="38" t="inlineStr">
+        <is>
+          <t>301 THIS -&gt; /low-blood-pressure-and-hair-loss/ (keep the winner: 79 clicks/90d vs 8, position 10.1 vs 22.8). Merge any unique content into the winner first. Redirect rule drafted in docs/seo/technical/OP-02-duplicate-redirects.md.</t>
+        </is>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="33" t="inlineStr">
@@ -64633,6 +64734,10 @@
       <c r="I255" s="38" t="n"/>
       <c r="J255" s="38" t="n"/>
     </row>
+    <row r="256"/>
+    <row r="257"/>
+    <row r="258"/>
+    <row r="259"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
OP-03: ready-to-paste fix for the 3 priority zero-click pages
Two-part fix per page, matching how Rank Math is already being used for
the redirects: (1) SEO Title + Meta Description rewrite via Rank Math's
per-post snippet editor - this is what actually competes with an AI
Overview for the click; (2) an additive self-assessment/CTA content
block near the top of the existing page, not a rewrite - these pages
already rank well, so the fix is giving a reason to click through, not
re-explaining the topic.

Exact copy provided for /can-hair-grow-back-after-thinning/ (the worst
case, pos 5.2 / 0.02% CTR), /hair-prp-price-in-pakistan/, and
/scalp-reduction-surgery/. Lighter guidance for the 3 lower-priority
post-op pages with a different CTA angle (WhatsApp post-op support
rather than a new consultation).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VmvRFCrr5iCSGjZGbzZndE
</commit_message>
<xml_diff>
--- a/docs/seo/DrRanaIrfanSEOIssueTracker.xlsx
+++ b/docs/seo/DrRanaIrfanSEOIssueTracker.xlsx
@@ -655,7 +655,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K1000"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6" customWidth="1" style="23" min="1" max="1"/>
     <col width="38" customWidth="1" style="23" min="2" max="2"/>
@@ -14446,7 +14446,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K1000"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6" customWidth="1" style="23" min="1" max="1"/>
     <col width="38" customWidth="1" style="23" min="2" max="2"/>
@@ -28141,7 +28141,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K1000"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="6" customWidth="1" style="23" min="1" max="1"/>
     <col width="38" customWidth="1" style="23" min="2" max="2"/>
@@ -42000,7 +42000,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:I331"/>
-  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="8" defaultColWidth="14.43" defaultRowHeight="15" customHeight="1"/>
   <cols>
     <col width="5" customWidth="1" style="23" min="1" max="1"/>
     <col width="34" customWidth="1" style="23" min="2" max="2"/>
@@ -56197,8 +56197,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" style="23" min="1" max="1"/>
     <col width="18" customWidth="1" style="23" min="2" max="2"/>
@@ -56638,6 +56638,43 @@
         </is>
       </c>
       <c r="G15" s="32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="130" customHeight="1" s="23">
+      <c r="A16" s="31" t="inlineStr">
+        <is>
+          <t>2026-10-02</t>
+        </is>
+      </c>
+      <c r="B16" s="31" t="inlineStr">
+        <is>
+          <t>On Page SEO Issue</t>
+        </is>
+      </c>
+      <c r="C16" s="31" t="inlineStr">
+        <is>
+          <t>OP-03 (fix walkthrough)</t>
+        </is>
+      </c>
+      <c r="D16" s="31" t="inlineStr">
+        <is>
+          <t>Wrote the actual field-by-field fix for the 3 priority zero-click pages, so the finding converts into something executable in wp-admin rather than staying analysis.</t>
+        </is>
+      </c>
+      <c r="E16" s="31" t="inlineStr">
+        <is>
+          <t>docs/seo/content/OP-03-fix-walkthrough.md: ready-to-paste SEO Title + Meta Description (via Rank Math's per-post snippet editor) and an on-page self-assessment/CTA block to add near the top (not a rewrite - these pages already rank well, so existing content stays, new content is additive) for /can-hair-grow-back-after-thinning/, /hair-prp-price-in-pakistan/, and /scalp-reduction-surgery/. Lighter guidance for the 3 lower-priority post-op pages, with a different CTA angle (WhatsApp post-op support, not a new consultation) since those readers have usually already had the procedure. Not applied - needs WordPress access.</t>
+        </is>
+      </c>
+      <c r="F16" s="31" t="inlineStr">
+        <is>
+          <t>docs/seo/content/OP-03-fix-walkthrough.md</t>
+        </is>
+      </c>
+      <c r="G16" s="32" t="inlineStr">
         <is>
           <t>No</t>
         </is>
@@ -56664,8 +56701,8 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J259"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
+  <dimension ref="A1:J255"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" style="23" min="1" max="1"/>
     <col width="10" customWidth="1" style="23" min="2" max="2"/>
@@ -64933,10 +64970,6 @@
       <c r="I255" s="38" t="n"/>
       <c r="J255" s="38" t="n"/>
     </row>
-    <row r="256"/>
-    <row r="257"/>
-    <row r="258"/>
-    <row r="259"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:J1"/>

</xml_diff>

<commit_message>
Upgrade confirmed credentials after user verified IMCAS profile
The user checked Dr. Rana Irfan's real IMCAS profile and shared its
content, which independently confirms two facts previously withheld
pending verification: President (2025) of HRSP, and - new - "first
non-American to serve as President of ABHRS". The latter is a stronger
press hook than anything in the original OFF-09 draft.

Rewrote the OFF-09 press pitch to lead with the "first non-American"
angle and marked both facts confirmed rather than bracketed. Upgraded
the OP-01 author bio box with the same two facts plus ABHRS Diplomate
status. Flagged the IMCAS profile itself as a candidate for OP-12's
Person schema sameAs list, pending confirmation of whether the page
actually links back to drranairfan.com - couldn't verify directly, this
environment blocks fetching imcas.com.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VmvRFCrr5iCSGjZGbzZndE
</commit_message>
<xml_diff>
--- a/docs/seo/DrRanaIrfanSEOIssueTracker.xlsx
+++ b/docs/seo/DrRanaIrfanSEOIssueTracker.xlsx
@@ -855,7 +855,7 @@
       <c r="J6" s="16" t="n"/>
       <c r="K6" s="14" t="inlineStr">
         <is>
-          <t>Drafted ready-to-use byline/medical-reviewer content in docs/seo/content/OP-01-author-bio-boxes.md: a full bio box + short 'Medically reviewed by' line for Dr. Rana Irfan using only confirmed credentials (Immediate Past President ABHRS, FISHRS, 25+ years, real ABHRS/ISHRS/social profile links). Dr. Uzma Irfan's bio is a placeholder only - no confirmed individual credentials for her exist in this engagement, so it's deliberately not filled in. Actual site-wide application needs WordPress/Elementor access this agent doesn't have, and should happen after the OP-02 blog audit (no point bylining a page that's about to be merged/deleted).</t>
+          <t>Drafted ready-to-use byline/medical-reviewer content in docs/seo/content/OP-01-author-bio-boxes.md: a full bio box + short 'Medically reviewed by' line for Dr. Rana Irfan using only confirmed credentials (Immediate Past President ABHRS, FISHRS, 25+ years, real ABHRS/ISHRS/social profile links). Dr. Uzma Irfan's bio is a placeholder only - no confirmed individual credentials for her exist in this engagement, so it's deliberately not filled in. Actual site-wide application needs WordPress/Elementor access this agent doesn't have, and should happen after the OP-02 blog audit (no point bylining a page that's about to be merged/deleted). | UPDATE 2026-10-06: bio upgraded with newly-confirmed facts (HRSP presidency, first non-American ABHRS President, ABHRS Diplomate status) via Dr. Irfan's real IMCAS profile, shared by the user. See updated docs/seo/content/OP-01-author-bio-boxes.md.</t>
         </is>
       </c>
     </row>
@@ -1364,7 +1364,11 @@
         </is>
       </c>
       <c r="J17" s="16" t="n"/>
-      <c r="K17" s="14" t="n"/>
+      <c r="K17" s="14" t="inlineStr">
+        <is>
+          <t>Candidate sameAs source found 2026-10-06: Dr. Irfan's IMCAS profile (imcas.com/en/profile/dr-rana-irfan-2) - real, well-populated bio confirming ABHRS Diplomate, first non-American ABHRS President, FISHRS, HRSP President (2025). NOT YET confirmed whether the page itself links out to drranairfan.com - checking with the user before adding to the sameAs list. Pending that, combine with the ABHRS/ISHRS profiles already confirmed in OFF-08 for the full Person schema sameAs array.</t>
+        </is>
+      </c>
     </row>
     <row r="18" ht="45.75" customHeight="1" s="23">
       <c r="A18" s="11" t="inlineStr">
@@ -15018,7 +15022,7 @@
       <c r="J14" s="16" t="n"/>
       <c r="K14" s="14" t="inlineStr">
         <is>
-          <t>Title confirmed by user (2026-09-11): Immediate Past President of ABHRS. Press pitch drafted in docs/seo/outreach/OFF-09-press-pitch.md, targeting Dawn/The News/Express Tribune/Business Recorder/Geo per this row's recommendation. Two claims in the draft (HRSP presidency, procedure count) are flagged as unconfirmed and bracketed for the clinic to verify or remove before sending - not asserted on my own authority. Needs clinic staff to pick a named editor contact per outlet and actually send it.</t>
+          <t>Title confirmed by user (2026-09-11): Immediate Past President of ABHRS. Press pitch drafted in docs/seo/outreach/OFF-09-press-pitch.md, targeting Dawn/The News/Express Tribune/Business Recorder/Geo per this row's recommendation. Two claims in the draft (HRSP presidency, procedure count) are flagged as unconfirmed and bracketed for the clinic to verify or remove before sending - not asserted on my own authority. Needs clinic staff to pick a named editor contact per outlet and actually send it. | UPDATE 2026-10-06: the two previously-unconfirmed facts (HRSP presidency, 'first non-American ABHRS President') are now confirmed via Dr. Irfan's real IMCAS profile (imcas.com/en/profile/dr-rana-irfan-2), shared directly by the user. Pitch rewritten to lead with the stronger 'first non-American' hook. See updated docs/seo/outreach/OFF-09-press-pitch.md.</t>
         </is>
       </c>
     </row>
@@ -56201,7 +56205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" style="23" min="1" max="1"/>
@@ -56716,6 +56720,43 @@
         </is>
       </c>
       <c r="G17" s="32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="160" customHeight="1" s="23">
+      <c r="A18" s="31" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B18" s="31" t="inlineStr">
+        <is>
+          <t>Off Page SEO Issue, On Page SEO Issue</t>
+        </is>
+      </c>
+      <c r="C18" s="31" t="inlineStr">
+        <is>
+          <t>OFF-09, OP-01, OP-12</t>
+        </is>
+      </c>
+      <c r="D18" s="31" t="inlineStr">
+        <is>
+          <t>Upgraded two credential claims from unconfirmed to confirmed after the user checked a real third-party source (Dr. Irfan's IMCAS profile), and evaluated that profile itself as a potential quality backlink/sameAs source.</t>
+        </is>
+      </c>
+      <c r="E18" s="31" t="inlineStr">
+        <is>
+          <t>User shared Dr. Rana Irfan's IMCAS (International Master Course on Aging Science - a real, long-established dermatology/aesthetic medicine conference organization) profile. It independently confirms two facts this agent had previously withheld pending verification: President (2025) of HRSP, and - new information - 'first non-American to serve as President of ABHRS', a stronger press hook than what was drafted. Updated docs/seo/outreach/OFF-09-press-pitch.md (rewritten to lead with the new hook) and docs/seo/content/OP-01-author-bio-boxes.md (bio upgraded) accordingly - both now cite real, confirmed facts rather than carrying CONFIRM placeholders for these two items. Flagged the IMCAS profile itself as a candidate for OP-12's Person schema sameAs list, pending confirmation from the user whether the page actually links back to drranairfan.com (could not verify directly - this environment blocks fetching imcas.com).</t>
+        </is>
+      </c>
+      <c r="F18" s="31" t="inlineStr">
+        <is>
+          <t>docs/seo/outreach/OFF-09-press-pitch.md; docs/seo/content/OP-01-author-bio-boxes.md; tracker rows OFF-09, OP-01, OP-12</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>

<commit_message>
Add IMCAS as a third OFF-08 target; clarify it's still valid for OP-12
User confirmed the IMCAS profile has no outbound website link. Added it
as a third outreach target in OFF-08 alongside ABHRS/ISHRS, with a note
to try self-service editing first (the page shows a "Sign in" option,
suggesting members may be able to edit their own profile) before
emailing IMCAS support.

Corrected the OP-12 framing: schema.org sameAs is a one-directional
assertion from the clinic's own site to corroborating profiles - it
doesn't require the target page to link back. The IMCAS profile is a
confirmed-good sameAs candidate regardless of whether the link-request
above succeeds; that's a separate, optional upgrade (would make it an
actual backlink too), not a precondition for using it in schema.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01VmvRFCrr5iCSGjZGbzZndE
</commit_message>
<xml_diff>
--- a/docs/seo/DrRanaIrfanSEOIssueTracker.xlsx
+++ b/docs/seo/DrRanaIrfanSEOIssueTracker.xlsx
@@ -1366,7 +1366,7 @@
       <c r="J17" s="16" t="n"/>
       <c r="K17" s="14" t="inlineStr">
         <is>
-          <t>Candidate sameAs source found 2026-10-06: Dr. Irfan's IMCAS profile (imcas.com/en/profile/dr-rana-irfan-2) - real, well-populated bio confirming ABHRS Diplomate, first non-American ABHRS President, FISHRS, HRSP President (2025). NOT YET confirmed whether the page itself links out to drranairfan.com - checking with the user before adding to the sameAs list. Pending that, combine with the ABHRS/ISHRS profiles already confirmed in OFF-08 for the full Person schema sameAs array.</t>
+          <t>Confirmed by the user (2026-10-06): the IMCAS profile (imcas.com/en/profile/dr-rana-irfan-2) has NO outbound link, but that doesn't block using it as a sameAs source - sameAs is a one-directional assertion from drranairfan.com's own schema pointing at corroborating profiles, it doesn't require the target page to link back. Confirmed candidate for the Person schema sameAs array alongside ABHRS and ISHRS (both from OFF-08). Separately, requesting IMCAS add a link (OFF-08) would make it a real backlink too, but that's a distinct, optional upgrade, not a requirement for using it in schema.</t>
         </is>
       </c>
     </row>
@@ -14973,7 +14973,7 @@
       <c r="J13" s="16" t="n"/>
       <c r="K13" s="14" t="inlineStr">
         <is>
-          <t>Verified via web search (2026-09-11) that both the ABHRS and ISHRS profiles are real and live: abhrs.org/directory/listing/rana-irfan-md and ishrs.org/doctor/594807/. Could not fetch either page directly to check the current outbound link (this environment blocks fetches to arbitrary external domains) so 'does it already link' is still unconfirmed. Drafted ready-to-send outreach emails for both in docs/seo/outreach/OFF-08-society-profile-links.md. HRSP/IBHRS/FACS profile URLs not yet located - same pattern applies once found. Needs clinic staff to actually send + confirm the link was added.</t>
+          <t>Verified via web search (2026-09-11) that both the ABHRS and ISHRS profiles are real and live: abhrs.org/directory/listing/rana-irfan-md and ishrs.org/doctor/594807/. Could not fetch either page directly to check the current outbound link (this environment blocks fetches to arbitrary external domains) so 'does it already link' is still unconfirmed. Drafted ready-to-send outreach emails for both in docs/seo/outreach/OFF-08-society-profile-links.md. HRSP/IBHRS/FACS profile URLs not yet located - same pattern applies once found. Needs clinic staff to actually send + confirm the link was added. | UPDATE 2026-10-06: added IMCAS (imcas.com/en/profile/dr-rana-irfan-2) as a third target - confirmed by the user to be a real, well-populated profile with NO website link currently. Drafted outreach + flagged that the page's 'Sign in' option suggests self-service editing may be possible, worth trying before emailing IMCAS support. See updated docs/seo/outreach/OFF-08-society-profile-links.md.</t>
         </is>
       </c>
     </row>
@@ -56205,7 +56205,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="12" customWidth="1" style="23" min="1" max="1"/>
@@ -56757,6 +56757,43 @@
         </is>
       </c>
       <c r="G18" s="32" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="140" customHeight="1" s="23">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>2026-10-06</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>Off Page SEO Issue, On Page SEO Issue</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>OFF-08, OP-12</t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="inlineStr">
+        <is>
+          <t>User confirmed the IMCAS profile has no website link. Added it as a third OFF-08 outreach target and clarified it's still valid for OP-12's Person schema regardless.</t>
+        </is>
+      </c>
+      <c r="E19" s="31" t="inlineStr">
+        <is>
+          <t>Drafted an outreach request to IMCAS (or self-service edit attempt first, since the page shows a 'Sign in' option) asking them to add the drranairfan.com link - same pattern as the existing ABHRS/ISHRS requests. Separately corrected the framing on OP-12: schema.org sameAs is a one-directional signal from the clinic's own site to corroborating profiles: it does not require the target page to link back, so the IMCAS profile is a confirmed-good sameAs candidate regardless of whether the outreach above succeeds. Updated docs/seo/outreach/OFF-08-society-profile-links.md and tracker rows OFF-08, OP-12.</t>
+        </is>
+      </c>
+      <c r="F19" s="31" t="inlineStr">
+        <is>
+          <t>docs/seo/outreach/OFF-08-society-profile-links.md; tracker rows OFF-08, OP-12</t>
+        </is>
+      </c>
+      <c r="G19" s="32" t="inlineStr">
         <is>
           <t>No</t>
         </is>

</xml_diff>